<commit_message>
Minor corrections and additions
</commit_message>
<xml_diff>
--- a/source_data/Entognatha_taxonomy_traits.xlsx
+++ b/source_data/Entognatha_taxonomy_traits.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronquist/dev/ms-repos-iba/paper-mg-insects/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E659F2B8-76EF-284E-AC9D-E975DBE34B06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62F701CA-F4FE-A544-83F4-CB150A7B691A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bellini et al 2023" sheetId="1" r:id="rId1"/>
@@ -1736,19 +1736,19 @@
   </si>
   <si>
     <t>Saprophagous</t>
-    <phoneticPr fontId="10"/>
+    <phoneticPr fontId="12"/>
   </si>
   <si>
     <t>Soil</t>
-    <phoneticPr fontId="10"/>
+    <phoneticPr fontId="12"/>
   </si>
   <si>
     <t>Plants</t>
-    <phoneticPr fontId="10"/>
+    <phoneticPr fontId="12"/>
   </si>
   <si>
     <t>Water</t>
-    <phoneticPr fontId="10"/>
+    <phoneticPr fontId="12"/>
   </si>
   <si>
     <t>Clade</t>
@@ -2825,9 +2825,6 @@
     <t>Sinentomata</t>
   </si>
   <si>
-    <t>Acerontomata</t>
-  </si>
-  <si>
     <t>Rhabdura</t>
   </si>
   <si>
@@ -3066,17 +3063,34 @@
   </si>
   <si>
     <t>HQ882816.1 is a human sequence</t>
+  </si>
+  <si>
+    <t>Acerentomata</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -3354,87 +3368,89 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlänk" xfId="1" builtinId="8"/>
@@ -12417,15 +12433,15 @@
         <v>466</v>
       </c>
       <c r="D1" s="35" t="s">
+        <v>678</v>
+      </c>
+      <c r="H1" s="11" t="s">
         <v>679</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>680</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="37" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B2" s="37">
         <v>0</v>
@@ -12484,7 +12500,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="37" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B6" s="37">
         <v>0</v>
@@ -12495,7 +12511,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="37" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B7" s="37">
         <v>0</v>
@@ -12506,7 +12522,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="37" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B8" s="37">
         <v>0</v>
@@ -12554,7 +12570,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="46" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B11" s="37"/>
       <c r="C11" s="37"/>
@@ -12575,7 +12591,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="37" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B13" s="37">
         <v>0</v>
@@ -12586,7 +12602,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="37" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B14" s="37">
         <v>0</v>
@@ -12678,7 +12694,7 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="44" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B21" s="37">
         <v>0</v>
@@ -12689,7 +12705,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="44" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B22" s="37">
         <v>0</v>
@@ -12700,7 +12716,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="44" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B23" s="37">
         <v>0</v>
@@ -12718,7 +12734,7 @@
         <v>2</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
       <c r="E24" s="49" t="s">
         <v>140</v>
@@ -12733,7 +12749,7 @@
         <v>2</v>
       </c>
       <c r="D25" s="37" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="E25" s="49" t="s">
         <v>64</v>
@@ -12787,7 +12803,7 @@
         <v>501</v>
       </c>
       <c r="H28" s="52" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
@@ -12821,7 +12837,7 @@
         <v>504</v>
       </c>
       <c r="H30" s="51" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
@@ -12860,13 +12876,13 @@
         <v>4440</v>
       </c>
       <c r="D33" t="s">
+        <v>613</v>
+      </c>
+      <c r="E33" t="s">
         <v>614</v>
       </c>
-      <c r="E33" t="s">
+      <c r="F33" t="s">
         <v>615</v>
-      </c>
-      <c r="F33" t="s">
-        <v>616</v>
       </c>
       <c r="G33" s="48" t="s">
         <v>11</v>
@@ -13623,7 +13639,7 @@
         <v>519</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="M1" s="11" t="s">
         <v>383</v>
@@ -13632,7 +13648,7 @@
         <v>514</v>
       </c>
       <c r="O1" s="11" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -13673,13 +13689,13 @@
         <v>521</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="N2" s="42" t="s">
         <v>542</v>
       </c>
       <c r="O2" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -13726,7 +13742,7 @@
         <v>525</v>
       </c>
       <c r="O3" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
@@ -13770,7 +13786,7 @@
         <v>527</v>
       </c>
       <c r="O4" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
@@ -13799,7 +13815,7 @@
         <v>521</v>
       </c>
       <c r="I5" s="42" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="J5" s="42" t="s">
         <v>516</v>
@@ -13811,13 +13827,13 @@
         <v>516</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="N5" s="42" t="s">
         <v>528</v>
       </c>
       <c r="O5" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
@@ -13864,7 +13880,7 @@
         <v>524</v>
       </c>
       <c r="O6" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
@@ -13905,13 +13921,13 @@
         <v>516</v>
       </c>
       <c r="M7" s="44" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="N7" s="42" t="s">
         <v>533</v>
       </c>
       <c r="O7" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
@@ -13952,13 +13968,13 @@
         <v>516</v>
       </c>
       <c r="M8" s="44" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="N8" s="42" t="s">
         <v>539</v>
       </c>
       <c r="O8" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
@@ -13999,13 +14015,13 @@
         <v>521</v>
       </c>
       <c r="M9" s="44" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="N9" s="42" t="s">
         <v>525</v>
       </c>
       <c r="O9" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
@@ -14049,7 +14065,7 @@
         <v>545</v>
       </c>
       <c r="O10" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
@@ -14096,7 +14112,7 @@
         <v>551</v>
       </c>
       <c r="O11" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
@@ -14140,7 +14156,7 @@
         <v>553</v>
       </c>
       <c r="O12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
@@ -14184,7 +14200,7 @@
         <v>555</v>
       </c>
       <c r="O13" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
@@ -14225,13 +14241,13 @@
         <v>516</v>
       </c>
       <c r="M14" s="44" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="N14" s="42" t="s">
         <v>558</v>
       </c>
       <c r="O14" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
@@ -14272,13 +14288,13 @@
         <v>516</v>
       </c>
       <c r="M15" s="44" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="N15" s="42" t="s">
         <v>561</v>
       </c>
       <c r="O15" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
@@ -14322,7 +14338,7 @@
         <v>571</v>
       </c>
       <c r="O16" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
@@ -14366,7 +14382,7 @@
         <v>564</v>
       </c>
       <c r="O17" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
@@ -14413,7 +14429,7 @@
         <v>569</v>
       </c>
       <c r="O18" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
@@ -14436,7 +14452,7 @@
         <v>563</v>
       </c>
       <c r="G19" s="44" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="H19" s="42" t="s">
         <v>516</v>
@@ -14454,10 +14470,10 @@
         <v>521</v>
       </c>
       <c r="N19" s="44" t="s">
+        <v>638</v>
+      </c>
+      <c r="O19" t="s">
         <v>639</v>
-      </c>
-      <c r="O19" t="s">
-        <v>640</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
@@ -14498,13 +14514,13 @@
         <v>521</v>
       </c>
       <c r="M20" s="44" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="N20" s="42" t="s">
         <v>571</v>
       </c>
       <c r="O20" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
@@ -14521,7 +14537,7 @@
         <v>378</v>
       </c>
       <c r="E21" s="44" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
       <c r="F21" s="42" t="s">
         <v>567</v>
@@ -14551,7 +14567,7 @@
         <v>574</v>
       </c>
       <c r="O21" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
@@ -14592,13 +14608,13 @@
         <v>516</v>
       </c>
       <c r="M22" s="44" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
       <c r="N22" s="42" t="s">
         <v>579</v>
       </c>
       <c r="O22" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
@@ -14645,7 +14661,7 @@
         <v>598</v>
       </c>
       <c r="O23" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.2">
@@ -14686,13 +14702,13 @@
         <v>521</v>
       </c>
       <c r="M24" s="44" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="N24" t="s">
         <v>595</v>
       </c>
       <c r="O24" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
@@ -14733,13 +14749,13 @@
         <v>521</v>
       </c>
       <c r="M25" s="44" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="N25" t="s">
         <v>583</v>
       </c>
       <c r="O25" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
@@ -14786,7 +14802,7 @@
         <v>587</v>
       </c>
       <c r="O26" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.2">
@@ -14827,13 +14843,13 @@
         <v>521</v>
       </c>
       <c r="M27" s="44" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="N27" t="s">
         <v>585</v>
       </c>
       <c r="O27" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.2">
@@ -14874,13 +14890,13 @@
         <v>516</v>
       </c>
       <c r="M28" s="44" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="N28" s="42" t="s">
         <v>591</v>
       </c>
       <c r="O28" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.2">
@@ -14903,7 +14919,7 @@
         <v>515</v>
       </c>
       <c r="G29" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H29" t="s">
         <v>516</v>
@@ -14921,10 +14937,10 @@
         <v>516</v>
       </c>
       <c r="M29" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="N29" s="44" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.2">
@@ -14947,7 +14963,7 @@
         <v>515</v>
       </c>
       <c r="G30" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H30" s="44" t="s">
         <v>521</v>
@@ -14965,10 +14981,10 @@
         <v>516</v>
       </c>
       <c r="M30" s="44" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="N30" s="44" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.2">
@@ -14991,13 +15007,13 @@
         <v>515</v>
       </c>
       <c r="G31" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H31" s="44" t="s">
         <v>521</v>
       </c>
       <c r="I31" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="J31" s="44" t="s">
         <v>516</v>
@@ -15009,10 +15025,10 @@
         <v>521</v>
       </c>
       <c r="M31" s="44" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="N31" s="44" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.2">
@@ -15035,13 +15051,13 @@
         <v>515</v>
       </c>
       <c r="G32" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H32" s="44" t="s">
         <v>521</v>
       </c>
       <c r="I32" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="J32" s="44" t="s">
         <v>516</v>
@@ -15053,18 +15069,18 @@
         <v>516</v>
       </c>
       <c r="M32" s="44" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="N32" s="44" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B33" s="42" t="s">
-        <v>602</v>
+      <c r="B33" s="54" t="s">
+        <v>682</v>
       </c>
       <c r="C33" s="42" t="s">
         <v>462</v>
@@ -15079,7 +15095,7 @@
         <v>515</v>
       </c>
       <c r="G33" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H33" t="s">
         <v>516</v>
@@ -15097,18 +15113,18 @@
         <v>516</v>
       </c>
       <c r="M33" s="44" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="N33" s="44" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B34" s="42" t="s">
-        <v>602</v>
+      <c r="B34" s="55" t="s">
+        <v>682</v>
       </c>
       <c r="C34" s="42" t="s">
         <v>9</v>
@@ -15123,7 +15139,7 @@
         <v>515</v>
       </c>
       <c r="G34" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H34" s="44" t="s">
         <v>516</v>
@@ -15141,18 +15157,18 @@
         <v>521</v>
       </c>
       <c r="M34" s="44" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="N34" s="44" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="42" t="s">
-        <v>602</v>
+      <c r="B35" s="55" t="s">
+        <v>682</v>
       </c>
       <c r="C35" s="42" t="s">
         <v>461</v>
@@ -15167,13 +15183,13 @@
         <v>515</v>
       </c>
       <c r="G35" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H35" t="s">
         <v>516</v>
       </c>
       <c r="I35" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="J35" t="s">
         <v>516</v>
@@ -15185,10 +15201,10 @@
         <v>516</v>
       </c>
       <c r="M35" s="44" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="N35" s="44" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
@@ -15196,7 +15212,7 @@
         <v>61</v>
       </c>
       <c r="B36" s="42" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C36" s="42" t="s">
         <v>62</v>
@@ -15211,7 +15227,7 @@
         <v>515</v>
       </c>
       <c r="G36" s="44" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="H36" s="44" t="s">
         <v>516</v>
@@ -15229,10 +15245,10 @@
         <v>521</v>
       </c>
       <c r="M36" s="44" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="N36" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
@@ -15240,10 +15256,10 @@
         <v>61</v>
       </c>
       <c r="B37" s="42" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C37" s="42" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>378</v>
@@ -15255,13 +15271,13 @@
         <v>515</v>
       </c>
       <c r="G37" s="44" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H37" s="44" t="s">
         <v>521</v>
       </c>
       <c r="I37" s="44" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="J37" s="44" t="s">
         <v>516</v>
@@ -15273,10 +15289,10 @@
         <v>516</v>
       </c>
       <c r="M37" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="N37" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
@@ -15284,7 +15300,7 @@
         <v>61</v>
       </c>
       <c r="B38" s="42" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C38" s="42" t="s">
         <v>458</v>
@@ -15299,13 +15315,13 @@
         <v>515</v>
       </c>
       <c r="G38" s="44" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H38" s="44" t="s">
         <v>521</v>
       </c>
       <c r="I38" s="44" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="J38" s="44" t="s">
         <v>516</v>
@@ -15317,10 +15333,10 @@
         <v>516</v>
       </c>
       <c r="M38" s="44" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="N38" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
@@ -15328,13 +15344,13 @@
         <v>61</v>
       </c>
       <c r="B39" s="42" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C39" s="44" t="s">
         <v>459</v>
       </c>
       <c r="D39" s="44" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="E39" s="44" t="s">
         <v>379</v>
@@ -15343,13 +15359,13 @@
         <v>515</v>
       </c>
       <c r="G39" s="44" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="H39" s="44" t="s">
         <v>521</v>
       </c>
       <c r="I39" s="44" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="J39" s="44" t="s">
         <v>516</v>
@@ -15361,10 +15377,10 @@
         <v>516</v>
       </c>
       <c r="M39" s="44" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="N39" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
@@ -15372,7 +15388,7 @@
         <v>61</v>
       </c>
       <c r="B40" s="42" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="C40" s="44" t="s">
         <v>460</v>
@@ -15387,7 +15403,7 @@
         <v>515</v>
       </c>
       <c r="G40" s="44" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="H40" s="44" t="s">
         <v>516</v>
@@ -15405,7 +15421,7 @@
         <v>516</v>
       </c>
       <c r="N40" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
@@ -15413,10 +15429,10 @@
         <v>61</v>
       </c>
       <c r="B41" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C41" s="42" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="D41" s="7" t="s">
         <v>384</v>
@@ -15425,10 +15441,10 @@
         <v>379</v>
       </c>
       <c r="F41" s="44" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="G41" s="44" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="H41" s="44" t="s">
         <v>521</v>
@@ -15446,10 +15462,10 @@
         <v>516</v>
       </c>
       <c r="M41" s="44" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="N41" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
@@ -15457,13 +15473,13 @@
         <v>61</v>
       </c>
       <c r="B42" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C42" s="42" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="D42" s="44" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="E42" s="44" t="s">
         <v>379</v>
@@ -15472,13 +15488,13 @@
         <v>515</v>
       </c>
       <c r="G42" s="44" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H42" s="44" t="s">
         <v>516</v>
       </c>
       <c r="I42" s="44" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="J42" s="44" t="s">
         <v>516</v>
@@ -15490,7 +15506,7 @@
         <v>516</v>
       </c>
       <c r="N42" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
@@ -15498,7 +15514,7 @@
         <v>61</v>
       </c>
       <c r="B43" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C43" s="42" t="s">
         <v>456</v>
@@ -15510,16 +15526,16 @@
         <v>379</v>
       </c>
       <c r="F43" s="44" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="G43" s="44" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="H43" s="44" t="s">
         <v>521</v>
       </c>
       <c r="I43" s="44" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="J43" s="44" t="s">
         <v>516</v>
@@ -15531,10 +15547,10 @@
         <v>516</v>
       </c>
       <c r="M43" s="44" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="N43" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
@@ -15542,7 +15558,7 @@
         <v>61</v>
       </c>
       <c r="B44" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C44" s="42" t="s">
         <v>138</v>
@@ -15557,7 +15573,7 @@
         <v>515</v>
       </c>
       <c r="G44" s="44" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="H44" s="44" t="s">
         <v>516</v>
@@ -15575,10 +15591,10 @@
         <v>521</v>
       </c>
       <c r="M44" s="44" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="N44" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
@@ -15586,13 +15602,13 @@
         <v>61</v>
       </c>
       <c r="B45" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="C45" s="42" t="s">
         <v>457</v>
       </c>
       <c r="D45" s="44" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="E45" s="44" t="s">
         <v>379</v>
@@ -15601,13 +15617,13 @@
         <v>515</v>
       </c>
       <c r="G45" s="44" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="H45" s="44" t="s">
         <v>516</v>
       </c>
       <c r="I45" s="44" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="J45" s="44" t="s">
         <v>516</v>
@@ -15619,10 +15635,10 @@
         <v>516</v>
       </c>
       <c r="M45" s="44" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="N45" s="44" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
@@ -15630,12 +15646,12 @@
     </row>
     <row r="49" spans="7:7" x14ac:dyDescent="0.2">
       <c r="G49" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="50" spans="7:7" x14ac:dyDescent="0.2">
       <c r="G50" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
   </sheetData>

</xml_diff>